<commit_message>
Lista: nova primeira mensagem, resposta para quem já tem sistema e 1º contato marcado
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PUuZ7qyCh49qQaUtVTCgXT
</commit_message>
<xml_diff>
--- a/saas-cobranca/LISTA-CLIENTES.xlsx
+++ b/saas-cobranca/LISTA-CLIENTES.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="626" uniqueCount="291">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="628" uniqueCount="293">
   <si>
     <t xml:space="preserve">Como usar esta planilha</t>
   </si>
@@ -124,27 +124,30 @@
     <t xml:space="preserve">Abrir</t>
   </si>
   <si>
-    <t xml:space="preserve">Falar com Edlaine. 5 a 16 anos, mensalidade R$80 a R$130.</t>
+    <t xml:space="preserve">Já tem sistema de cobrança (respondeu em 20/10/2026).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sem interesse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ver</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Escola de Futebol Coach Pro Arena</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jundiaí</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(11) 99962-0007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contato de guia local (sem data).</t>
   </si>
   <si>
     <t xml:space="preserve">Não contatado</t>
   </si>
   <si>
-    <t xml:space="preserve">Ver</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Escola de Futebol Coach Pro Arena</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jundiaí</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(11) 99962-0007</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Contato de guia local (sem data).</t>
-  </si>
-  <si>
     <t xml:space="preserve">Escola de Futebol MBrasil</t>
   </si>
   <si>
@@ -811,9 +814,6 @@
     <t xml:space="preserve">Fechou (cliente)</t>
   </si>
   <si>
-    <t xml:space="preserve">Sem interesse</t>
-  </si>
-  <si>
     <t xml:space="preserve">Número errado</t>
   </si>
   <si>
@@ -841,7 +841,7 @@
     <t xml:space="preserve">1. Primeira mensagem</t>
   </si>
   <si>
-    <t xml:space="preserve">Oi, tudo bem? Encontrei vocês pesquisando [tipo] em [cidade] e curti muito o trabalho! Pergunta rápida: vocês ainda cobram as mensalidades um por um no WhatsApp?
+    <t xml:space="preserve">Oi, tudo bem? Meu nome é [seu nome], eu ajudo escolinhas e academias a cobrar mensalidade de forma automática pelo WhatsApp. Vi o trabalho de vocês em [cidade] e queria saber: hoje vocês têm problema com aluno atrasando a mensalidade?
 (O botão "Abrir" da aba Clientes já manda essa mensagem pronta.)</t>
   </si>
   <si>
@@ -893,6 +893,12 @@
   </si>
   <si>
     <t xml:space="preserve">O banco gera o Pix, mas não manda a cobrança no WhatsApp de cada aluno, não lembra quem atrasou e não mostra a lista de quem deve. O sistema faz isso sozinho.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Objeção: "já temos sistema"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Que bom, obrigado pelo retorno! Só uma curiosidade: qual sistema vocês usam? Ele manda a cobrança sozinho no WhatsApp dos pais? Se um dia precisar de algo mais simples ou mais barato, fico à disposição.</t>
   </si>
   <si>
     <t xml:space="preserve">Objeção: "vou pensar"</t>
@@ -1156,11 +1162,19 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="12">
+  <dxfs count="13">
     <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FF1E7449"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFEDEDED"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -1736,7 +1750,7 @@
         <v>39</v>
       </c>
       <c r="L3" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M3" s="8"/>
       <c r="N3" s="6"/>
@@ -1756,7 +1770,7 @@
         <v>26</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>37</v>
@@ -1766,17 +1780,17 @@
       </c>
       <c r="G4" s="6"/>
       <c r="H4" s="5" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="I4" s="7" t="s">
         <v>32</v>
       </c>
       <c r="J4" s="6"/>
       <c r="K4" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="L4" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M4" s="8"/>
       <c r="N4" s="6"/>
@@ -1796,31 +1810,31 @@
         <v>26</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I5" s="7" t="s">
         <v>32</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="K5" s="6" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="L5" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M5" s="8"/>
       <c r="N5" s="6"/>
@@ -1837,34 +1851,34 @@
         <v>25</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="I6" s="7" t="s">
         <v>32</v>
       </c>
       <c r="J6" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="K6" s="6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="L6" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M6" s="8"/>
       <c r="N6" s="6"/>
@@ -1881,34 +1895,34 @@
         <v>25</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F7" s="5" t="s">
         <v>29</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="I7" s="7" t="s">
         <v>32</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="K7" s="6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="L7" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M7" s="8"/>
       <c r="N7" s="6"/>
@@ -1925,32 +1939,32 @@
         <v>25</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F8" s="5" t="s">
         <v>29</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I8" s="7" t="s">
         <v>32</v>
       </c>
       <c r="J8" s="6"/>
       <c r="K8" s="6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="L8" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M8" s="8"/>
       <c r="N8" s="6"/>
@@ -1967,30 +1981,30 @@
         <v>25</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F9" s="5" t="s">
         <v>29</v>
       </c>
       <c r="G9" s="6"/>
       <c r="H9" s="5" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="I9" s="7" t="s">
         <v>32</v>
       </c>
       <c r="J9" s="6"/>
       <c r="K9" s="6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="L9" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M9" s="8"/>
       <c r="N9" s="6"/>
@@ -2007,32 +2021,32 @@
         <v>25</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F10" s="5" t="s">
         <v>29</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="I10" s="7" t="s">
         <v>32</v>
       </c>
       <c r="J10" s="6"/>
       <c r="K10" s="6" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="L10" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M10" s="8"/>
       <c r="N10" s="6"/>
@@ -2049,34 +2063,34 @@
         <v>25</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F11" s="5" t="s">
         <v>29</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="I11" s="7" t="s">
         <v>32</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="K11" s="6" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="L11" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M11" s="8"/>
       <c r="N11" s="6"/>
@@ -2093,34 +2107,34 @@
         <v>25</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="I12" s="7" t="s">
         <v>32</v>
       </c>
       <c r="J12" s="6" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="K12" s="6" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="L12" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M12" s="8"/>
       <c r="N12" s="6"/>
@@ -2137,32 +2151,32 @@
         <v>25</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="G13" s="6"/>
       <c r="H13" s="5" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="I13" s="7" t="s">
         <v>32</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="K13" s="6" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="L13" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M13" s="8"/>
       <c r="N13" s="6"/>
@@ -2179,32 +2193,32 @@
         <v>25</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="G14" s="6"/>
       <c r="H14" s="5" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="I14" s="7" t="s">
         <v>32</v>
       </c>
       <c r="J14" s="6" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="K14" s="6" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="L14" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M14" s="8"/>
       <c r="N14" s="6"/>
@@ -2221,30 +2235,30 @@
         <v>25</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="G15" s="6"/>
       <c r="H15" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="I15" s="7" t="s">
         <v>32</v>
       </c>
       <c r="J15" s="6"/>
       <c r="K15" s="6" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="L15" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M15" s="8"/>
       <c r="N15" s="6"/>
@@ -2261,30 +2275,30 @@
         <v>25</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="G16" s="6"/>
       <c r="H16" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="I16" s="7" t="s">
         <v>32</v>
       </c>
       <c r="J16" s="6"/>
       <c r="K16" s="6" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="L16" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M16" s="8"/>
       <c r="N16" s="6"/>
@@ -2301,32 +2315,32 @@
         <v>25</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="G17" s="6"/>
       <c r="H17" s="5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="I17" s="7" t="s">
         <v>32</v>
       </c>
       <c r="J17" s="6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="K17" s="6" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="L17" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M17" s="8"/>
       <c r="N17" s="6"/>
@@ -2343,30 +2357,30 @@
         <v>25</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="G18" s="6"/>
       <c r="H18" s="5" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="I18" s="7" t="s">
         <v>32</v>
       </c>
       <c r="J18" s="6"/>
       <c r="K18" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="L18" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M18" s="8"/>
       <c r="N18" s="6"/>
@@ -2383,34 +2397,34 @@
         <v>25</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="I19" s="7" t="s">
         <v>32</v>
       </c>
       <c r="J19" s="6" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="K19" s="6" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="L19" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M19" s="8"/>
       <c r="N19" s="6"/>
@@ -2427,34 +2441,34 @@
         <v>25</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="I20" s="7" t="s">
         <v>32</v>
       </c>
       <c r="J20" s="6" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="K20" s="6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="L20" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M20" s="8"/>
       <c r="N20" s="6"/>
@@ -2471,32 +2485,32 @@
         <v>25</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G21" s="6"/>
       <c r="H21" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="I21" s="7" t="s">
         <v>32</v>
       </c>
       <c r="J21" s="6" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="K21" s="6" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="L21" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M21" s="8"/>
       <c r="N21" s="6"/>
@@ -2513,32 +2527,32 @@
         <v>25</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G22" s="6"/>
       <c r="H22" s="5" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="I22" s="7" t="s">
         <v>32</v>
       </c>
       <c r="J22" s="6" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="K22" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="L22" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M22" s="8"/>
       <c r="N22" s="6"/>
@@ -2555,34 +2569,34 @@
         <v>25</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G23" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="I23" s="7" t="s">
         <v>32</v>
       </c>
       <c r="J23" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K23" s="6" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="L23" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M23" s="8"/>
       <c r="N23" s="6"/>
@@ -2599,34 +2613,34 @@
         <v>25</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="I24" s="7" t="s">
         <v>32</v>
       </c>
       <c r="J24" s="6" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="K24" s="6" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L24" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M24" s="8"/>
       <c r="N24" s="6"/>
@@ -2643,32 +2657,32 @@
         <v>25</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G25" s="6"/>
       <c r="H25" s="5" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="I25" s="7" t="s">
         <v>32</v>
       </c>
       <c r="J25" s="6" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="K25" s="6" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="L25" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M25" s="8"/>
       <c r="N25" s="6"/>
@@ -2685,34 +2699,34 @@
         <v>25</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="I26" s="7" t="s">
         <v>32</v>
       </c>
       <c r="J26" s="6" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="K26" s="6" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="L26" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M26" s="8"/>
       <c r="N26" s="6"/>
@@ -2729,34 +2743,34 @@
         <v>25</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="G27" s="6" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="I27" s="7" t="s">
         <v>32</v>
       </c>
       <c r="J27" s="6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="K27" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="L27" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M27" s="8"/>
       <c r="N27" s="6"/>
@@ -2773,34 +2787,34 @@
         <v>25</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G28" s="6" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="I28" s="7" t="s">
         <v>32</v>
       </c>
       <c r="J28" s="6" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="K28" s="6" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="L28" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M28" s="8"/>
       <c r="N28" s="6"/>
@@ -2817,34 +2831,34 @@
         <v>25</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G29" s="6" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="H29" s="5" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I29" s="7" t="s">
         <v>32</v>
       </c>
       <c r="J29" s="6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="K29" s="6" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="L29" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M29" s="8"/>
       <c r="N29" s="6"/>
@@ -2861,32 +2875,32 @@
         <v>25</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F30" s="5" t="s">
         <v>29</v>
       </c>
       <c r="G30" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="I30" s="7" t="s">
         <v>32</v>
       </c>
       <c r="J30" s="6"/>
       <c r="K30" s="6" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="L30" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M30" s="8"/>
       <c r="N30" s="6"/>
@@ -2903,30 +2917,30 @@
         <v>25</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F31" s="5" t="s">
         <v>29</v>
       </c>
       <c r="G31" s="6"/>
       <c r="H31" s="5" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="I31" s="7" t="s">
         <v>32</v>
       </c>
       <c r="J31" s="6"/>
       <c r="K31" s="6" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="L31" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M31" s="8"/>
       <c r="N31" s="6"/>
@@ -2943,30 +2957,30 @@
         <v>25</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F32" s="5" t="s">
         <v>29</v>
       </c>
       <c r="G32" s="6"/>
       <c r="H32" s="5" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="I32" s="7" t="s">
         <v>32</v>
       </c>
       <c r="J32" s="6"/>
       <c r="K32" s="6" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="L32" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M32" s="8"/>
       <c r="N32" s="6"/>
@@ -2983,32 +2997,32 @@
         <v>25</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F33" s="5" t="s">
         <v>29</v>
       </c>
       <c r="G33" s="6" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="H33" s="5" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="I33" s="7" t="s">
         <v>32</v>
       </c>
       <c r="J33" s="6"/>
       <c r="K33" s="6" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="L33" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M33" s="8"/>
       <c r="N33" s="6"/>
@@ -3025,34 +3039,34 @@
         <v>25</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F34" s="5" t="s">
         <v>29</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="H34" s="5" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="I34" s="7" t="s">
         <v>32</v>
       </c>
       <c r="J34" s="6" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="K34" s="6" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="L34" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M34" s="8"/>
       <c r="N34" s="6"/>
@@ -3066,35 +3080,35 @@
         <v>34</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C35" s="5" t="s">
         <v>26</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F35" s="5" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="G35" s="6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="H35" s="5" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="I35" s="5" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="J35" s="6"/>
       <c r="K35" s="6" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="L35" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M35" s="8"/>
       <c r="N35" s="6"/>
@@ -3108,37 +3122,37 @@
         <v>35</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C36" s="5" t="s">
         <v>26</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F36" s="5" t="s">
         <v>29</v>
       </c>
       <c r="G36" s="6" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="H36" s="5" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I36" s="5" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="J36" s="6" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="K36" s="6" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="L36" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M36" s="8"/>
       <c r="N36" s="6"/>
@@ -3152,33 +3166,33 @@
         <v>36</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F37" s="5" t="s">
         <v>29</v>
       </c>
       <c r="G37" s="6"/>
       <c r="H37" s="5" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="I37" s="5" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="J37" s="6"/>
       <c r="K37" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="L37" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M37" s="8"/>
       <c r="N37" s="6"/>
@@ -3192,37 +3206,37 @@
         <v>37</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F38" s="5" t="s">
         <v>29</v>
       </c>
       <c r="G38" s="6" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="H38" s="5" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="I38" s="5" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="J38" s="6" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="K38" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="L38" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M38" s="8"/>
       <c r="N38" s="6"/>
@@ -3236,37 +3250,37 @@
         <v>38</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="E39" s="5" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="F39" s="5" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="G39" s="6" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="H39" s="5" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I39" s="5" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="J39" s="6" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="K39" s="6" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="L39" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M39" s="8"/>
       <c r="N39" s="6"/>
@@ -3280,37 +3294,37 @@
         <v>39</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="F40" s="5" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="G40" s="6" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="H40" s="5" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I40" s="5" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="J40" s="6" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="K40" s="6" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="L40" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M40" s="8"/>
       <c r="N40" s="6"/>
@@ -3324,37 +3338,37 @@
         <v>40</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="E41" s="5" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F41" s="5" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G41" s="6" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="H41" s="5" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I41" s="5" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="J41" s="6" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="K41" s="6" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="L41" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M41" s="8"/>
       <c r="N41" s="6"/>
@@ -3368,37 +3382,37 @@
         <v>41</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F42" s="5" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G42" s="6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H42" s="5" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I42" s="5" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="J42" s="6" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="K42" s="6" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="L42" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M42" s="8"/>
       <c r="N42" s="6"/>
@@ -3412,37 +3426,37 @@
         <v>42</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="E43" s="5" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F43" s="5" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G43" s="6" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="H43" s="5" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I43" s="5" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="J43" s="6" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="K43" s="6" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="L43" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M43" s="8"/>
       <c r="N43" s="6"/>
@@ -3456,35 +3470,35 @@
         <v>43</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="E44" s="5" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F44" s="5" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="G44" s="6"/>
       <c r="H44" s="5" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="I44" s="5" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="J44" s="6" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="K44" s="6" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="L44" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M44" s="8"/>
       <c r="N44" s="6"/>
@@ -3498,37 +3512,37 @@
         <v>44</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="E45" s="5" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F45" s="5" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="G45" s="6" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="H45" s="5" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I45" s="5" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="J45" s="6" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="K45" s="6" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="L45" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M45" s="8"/>
       <c r="N45" s="6"/>
@@ -3542,37 +3556,37 @@
         <v>45</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E46" s="5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F46" s="5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G46" s="6" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="H46" s="5" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="I46" s="7" t="s">
         <v>32</v>
       </c>
       <c r="J46" s="6" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="K46" s="6" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="L46" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M46" s="8"/>
       <c r="N46" s="6"/>
@@ -3586,37 +3600,37 @@
         <v>46</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="E47" s="5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F47" s="5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G47" s="6" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="H47" s="5" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="I47" s="5" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="J47" s="6" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="K47" s="6" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="L47" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M47" s="8"/>
       <c r="N47" s="6"/>
@@ -3630,35 +3644,35 @@
         <v>47</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D48" s="6" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="E48" s="5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F48" s="5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G48" s="6" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="H48" s="5" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="I48" s="5" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="J48" s="6"/>
       <c r="K48" s="6" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="L48" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M48" s="8"/>
       <c r="N48" s="6"/>
@@ -3672,37 +3686,37 @@
         <v>48</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="E49" s="5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F49" s="5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G49" s="6" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="H49" s="5" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I49" s="5" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="J49" s="6" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="K49" s="6" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="L49" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M49" s="8"/>
       <c r="N49" s="6"/>
@@ -3716,33 +3730,33 @@
         <v>49</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D50" s="6" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E50" s="5" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F50" s="5" t="s">
         <v>29</v>
       </c>
       <c r="G50" s="6"/>
       <c r="H50" s="5" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="I50" s="5" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="J50" s="6"/>
       <c r="K50" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="L50" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="M50" s="8"/>
       <c r="N50" s="6"/>
@@ -3753,35 +3767,35 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:P50">
-    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
       <formula>$L2="Fechou (cliente)"</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
       <formula>$L2="Teste grátis"</formula>
     </cfRule>
-    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+    <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>$L2="Respondeu"</formula>
     </cfRule>
-    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+    <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
       <formula>$L2="Vídeo/demo enviado"</formula>
     </cfRule>
-    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+    <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
       <formula>$L2="Mensagem enviada"</formula>
     </cfRule>
-    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
+    <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
       <formula>$L2="Sem interesse"</formula>
     </cfRule>
-    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="9">
+    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
       <formula>$L2="Número errado"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B2:B50">
-    <cfRule type="expression" priority="9" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
+    <cfRule type="expression" priority="9" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
       <formula>$B2="A"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O2:O50">
-    <cfRule type="expression" priority="10" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
+    <cfRule type="expression" priority="10" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>AND($O2&lt;&gt;"",$O2&lt;=TODAY(),$L2&lt;&gt;"Fechou (cliente)",$L2&lt;&gt;"Sem interesse")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3906,12 +3920,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3919,31 +3933,31 @@
         <v>11</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D4" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>258</v>
+      </c>
+      <c r="F4" s="11" t="s">
+        <v>259</v>
+      </c>
+      <c r="G4" s="11" t="s">
+        <v>260</v>
+      </c>
+      <c r="H4" s="11" t="s">
+        <v>261</v>
+      </c>
+      <c r="I4" s="11" t="s">
+        <v>262</v>
+      </c>
+      <c r="J4" s="11" t="s">
         <v>34</v>
-      </c>
-      <c r="E4" s="11" t="s">
-        <v>257</v>
-      </c>
-      <c r="F4" s="11" t="s">
-        <v>258</v>
-      </c>
-      <c r="G4" s="11" t="s">
-        <v>259</v>
-      </c>
-      <c r="H4" s="11" t="s">
-        <v>260</v>
-      </c>
-      <c r="I4" s="11" t="s">
-        <v>261</v>
-      </c>
-      <c r="J4" s="11" t="s">
-        <v>262</v>
       </c>
       <c r="K4" s="11" t="s">
         <v>263</v>
@@ -3963,7 +3977,7 @@
       </c>
       <c r="D5" s="13" t="n">
         <f aca="false">COUNTIFS(Clientes!$C:$C,$A5,Clientes!$L:$L,D$4)</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E5" s="13" t="n">
         <f aca="false">COUNTIFS(Clientes!$C:$C,$A5,Clientes!$L:$L,E$4)</f>
@@ -3987,7 +4001,7 @@
       </c>
       <c r="J5" s="13" t="n">
         <f aca="false">COUNTIFS(Clientes!$C:$C,$A5,Clientes!$L:$L,J$4)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K5" s="13" t="n">
         <f aca="false">COUNTIFS(Clientes!$C:$C,$A5,Clientes!$L:$L,K$4)</f>
@@ -3996,7 +4010,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B6" s="13" t="n">
         <f aca="false">COUNTIF(Clientes!$C:$C,$A6)</f>
@@ -4041,7 +4055,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B7" s="13" t="n">
         <f aca="false">COUNTIF(Clientes!$C:$C,$A7)</f>
@@ -4086,7 +4100,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B8" s="13" t="n">
         <f aca="false">COUNTIF(Clientes!$C:$C,$A8)</f>
@@ -4131,7 +4145,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B9" s="13" t="n">
         <f aca="false">COUNTIF(Clientes!$C:$C,$A9)</f>
@@ -4176,7 +4190,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B10" s="13" t="n">
         <f aca="false">COUNTIF(Clientes!$C:$C,$A10)</f>
@@ -4221,7 +4235,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="B11" s="14" t="n">
         <f aca="false">SUM(B5:B10)</f>
@@ -4233,7 +4247,7 @@
       </c>
       <c r="D11" s="14" t="n">
         <f aca="false">SUM(D5:D10)</f>
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E11" s="14" t="n">
         <f aca="false">SUM(E5:E10)</f>
@@ -4257,7 +4271,7 @@
       </c>
       <c r="J11" s="14" t="n">
         <f aca="false">SUM(J5:J10)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K11" s="14" t="n">
         <f aca="false">SUM(K5:K10)</f>
@@ -4270,7 +4284,7 @@
       </c>
       <c r="B13" s="16" t="n">
         <f aca="false">IFERROR((F11+G11+H11+I11+J11)/(B11-D11-K11),0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C13" s="17" t="s">
         <v>265</v>
@@ -4321,7 +4335,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
@@ -4333,7 +4347,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="20" t="s">
         <v>271</v>
       </c>
@@ -4405,12 +4419,20 @@
         <v>288</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="20" t="s">
         <v>289</v>
       </c>
       <c r="B12" s="21" t="s">
         <v>290</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="20" t="s">
+        <v>291</v>
+      </c>
+      <c r="B13" s="21" t="s">
+        <v>292</v>
       </c>
     </row>
   </sheetData>

</xml_diff>